<commit_message>
docs: mise à jour du planning, du rapport et des diagrammes
</commit_message>
<xml_diff>
--- a/doc/GAMEZ_Planning.xlsx
+++ b/doc/GAMEZ_Planning.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/thibaudfrederic_gamez_studentfr_ch/Documents/TPI/tpi2026-codementor/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:1_{A9F33111-F1CD-44EA-A64F-CD2C69F07527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DEA98A6C-95FC-4039-AA67-4A3487CCD557}"/>
+  <xr:revisionPtr revIDLastSave="92" documentId="13_ncr:1_{A9F33111-F1CD-44EA-A64F-CD2C69F07527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EDE35340-B8DE-40CD-9BAA-713B1CAED8B3}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planning EMF-EPAI" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Planning EMF-EPAI'!$A$1:$GU$43</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Planning EMF-EPAI'!$1:$5,'Planning EMF-EPAI'!$A:$C</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Planning EMF-EPAI'!$A$1:$GU$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="71">
   <si>
     <t xml:space="preserve">Projet : CodeMentor                        </t>
   </si>
@@ -1938,7 +1938,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:GV59"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="50.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.7109375" style="3" customWidth="1"/>
@@ -4439,7 +4439,7 @@
         <v>28</v>
       </c>
       <c r="B11" s="43" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C11" s="35"/>
       <c r="D11" s="59"/>
@@ -4654,7 +4654,9 @@
       <c r="A12" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="43"/>
+      <c r="B12" s="43" t="s">
+        <v>23</v>
+      </c>
       <c r="C12" s="35"/>
       <c r="D12" s="59"/>
       <c r="E12" s="57"/>
@@ -4866,7 +4868,9 @@
       <c r="A13" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="43"/>
+      <c r="B13" s="43" t="s">
+        <v>23</v>
+      </c>
       <c r="C13" s="35"/>
       <c r="D13" s="5"/>
       <c r="E13" s="6"/>
@@ -5490,7 +5494,9 @@
       <c r="A16" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="43"/>
+      <c r="B16" s="43" t="s">
+        <v>23</v>
+      </c>
       <c r="C16" s="35"/>
       <c r="D16" s="59"/>
       <c r="E16" s="57"/>
@@ -5702,7 +5708,9 @@
       <c r="A17" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="43"/>
+      <c r="B17" s="43" t="s">
+        <v>23</v>
+      </c>
       <c r="C17" s="35"/>
       <c r="D17" s="59"/>
       <c r="E17" s="57"/>
@@ -5912,7 +5920,9 @@
       <c r="A18" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="43"/>
+      <c r="B18" s="43" t="s">
+        <v>23</v>
+      </c>
       <c r="C18" s="35"/>
       <c r="D18" s="59"/>
       <c r="E18" s="57"/>
@@ -5954,8 +5964,12 @@
       <c r="AO18" s="71"/>
       <c r="AP18" s="57"/>
       <c r="AQ18" s="58"/>
-      <c r="AR18" s="59"/>
-      <c r="AS18" s="57"/>
+      <c r="AR18" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="AS18" s="57" t="s">
+        <v>24</v>
+      </c>
       <c r="AT18" s="57"/>
       <c r="AU18" s="57"/>
       <c r="AV18" s="57"/>
@@ -6120,7 +6134,9 @@
       <c r="A19" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="43"/>
+      <c r="B19" s="43" t="s">
+        <v>26</v>
+      </c>
       <c r="C19" s="35"/>
       <c r="D19" s="59"/>
       <c r="E19" s="57"/>
@@ -6164,7 +6180,9 @@
       <c r="AQ19" s="58"/>
       <c r="AR19" s="59"/>
       <c r="AS19" s="57"/>
-      <c r="AT19" s="57"/>
+      <c r="AT19" s="57" t="s">
+        <v>24</v>
+      </c>
       <c r="AU19" s="57"/>
       <c r="AV19" s="57"/>
       <c r="AW19" s="57"/>
@@ -6373,7 +6391,9 @@
       <c r="AR20" s="59"/>
       <c r="AS20" s="57"/>
       <c r="AT20" s="57"/>
-      <c r="AU20" s="57"/>
+      <c r="AU20" s="57" t="s">
+        <v>24</v>
+      </c>
       <c r="AV20" s="57"/>
       <c r="AW20" s="57"/>
       <c r="AX20" s="57"/>
@@ -14264,9 +14284,13 @@
       <c r="AN58" s="97"/>
       <c r="AO58" s="94"/>
       <c r="AP58" s="94"/>
-      <c r="AQ58" s="95"/>
+      <c r="AQ58" s="95" t="s">
+        <v>24</v>
+      </c>
       <c r="AR58" s="96"/>
-      <c r="AS58" s="94"/>
+      <c r="AS58" s="94" t="s">
+        <v>24</v>
+      </c>
       <c r="AT58" s="94"/>
       <c r="AU58" s="94"/>
       <c r="AV58" s="97"/>

</xml_diff>